<commit_message>
Remove all pay-on-delivery wording
Deck cover, payment card and closing page rebuilt for payment in
advance; SOPs, Clients and Finance sheets updated (no pro rata
invoices); SOP PDF re-exported.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012aVsoCbqH8naSiNgykD1Dt
</commit_message>
<xml_diff>
--- a/yontro-sheets/Yontro Finance & Growth (Confidential).xlsx
+++ b/yontro-sheets/Yontro Finance & Growth (Confidential).xlsx
@@ -83,7 +83,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Invoice date + 5 days (service agreement)</t>
+          <t xml:space="preserve">Invoice date + 7 days: paid in advance, before the service month starts</t>
         </r>
       </text>
     </comment>
@@ -653,10 +653,10 @@
     <t xml:space="preserve">UAE standard VAT rate. Only charge it if Yontro is VAT-registered</t>
   </si>
   <si>
-    <t xml:space="preserve">Days to pay an invoice</t>
+    <t xml:space="preserve">Days from invoice to due date</t>
   </si>
   <si>
-    <t xml:space="preserve">Service agreement clause 4</t>
+    <t xml:space="preserve">Service Agreement: invoiced 7 days before the month starts, paid before it starts</t>
   </si>
   <si>
     <t xml:space="preserve">Package</t>
@@ -21673,7 +21673,7 @@
       </c>
       <c r="J2" s="16" t="n">
         <f aca="false">IF(B2="","",B2+Settings!$B$13)</f>
-        <v>46349</v>
+        <v>46351</v>
       </c>
       <c r="K2" s="8" t="n">
         <v>46344</v>
@@ -56288,7 +56288,7 @@
         <v>117</v>
       </c>
       <c r="B13" s="27" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C13" s="6" t="s">
         <v>118</v>

</xml_diff>